<commit_message>
Update session details and moderator names for Recife Tórax 2026
- Added new moderators for various sessions, including Ana Rita Carvalho for Mesa 1 and José Fernando Prado for Mesa 2.
- Revised speaker names and details in the schedule, ensuring accurate representation across HTML and CSV files.
- Updated session descriptions and timings for clarity, including changes to moderator names and speaker affiliations.
</commit_message>
<xml_diff>
--- a/recifetorax2026/schedule/programacao-preliminar.xlsx
+++ b/recifetorax2026/schedule/programacao-preliminar.xlsx
@@ -66,7 +66,7 @@
   <si>
     <t xml:space="preserve">Mesa 1: Atualização em Fatores de Risco e Diagnóstico Precoce 
 Presidente: Alfredo Leite 
-Moderadores:   Leonardo Pontual ,  Antônio Douglas</t>
+Moderadores:   Leonardo Pontual ,  Antônio Douglas, Ana Rita Carvalho </t>
   </si>
   <si>
     <t xml:space="preserve">08:30 - 08:45 
@@ -121,7 +121,7 @@
   <si>
     <t xml:space="preserve">Mesa 2: Doença localizada
 Presidente: Bruno Pacheco 
-Moderadores:  Thiago Apolinario,  Ricardo Machado, Gustavo Ferreira </t>
+Moderadores:  José Fernando Prado,  Ricardo Machado, Gustavo Ferreira </t>
   </si>
   <si>
     <t xml:space="preserve">CASO CLINICO </t>
@@ -148,7 +148,7 @@
   <si>
     <t xml:space="preserve">Mesa 3 : DESAFIOS NA CIRURGIA 
 Presidente:  Tomás Béder 
-Moderadores:   Eriberto,  Paula Abreu e Lima,  Franceane</t>
+Moderadores:   Eriberto,  Paula Abreu e Lima,  France Anne Reinaldo </t>
   </si>
   <si>
     <t xml:space="preserve">10:40 - 10:55
@@ -182,7 +182,7 @@
     <t xml:space="preserve">SIMPOSIO SATELITE ASTRAZENECA - Doença Iressecavel - PACIFIC/LAURA</t>
   </si>
   <si>
-    <t xml:space="preserve">Victor Gondim </t>
+    <t xml:space="preserve">Victor Gondim - RJ</t>
   </si>
   <si>
     <t xml:space="preserve">12:15- 13:15
@@ -196,9 +196,19 @@
 (40 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">Mesa 4: Doença localmente - Irressecável  e Oligometastatica 
+    <r>
+      <t xml:space="preserve">Mesa 4: Doença localmente - Irressecável  e Oligometastatica 
 Presidente: Petrúcio Sarmento 
-Moderadores:  Victor Gondim, Thiago Darlan</t>
+Moderadores:  Victor Gondim, Thiago Darlan, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="64"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve">Suzane Leite</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">13:15 - 13:35
@@ -222,7 +232,7 @@
     <t xml:space="preserve">SIMPÓSIO SATÉLITE JOHNSON  - Anticorpos biespecíficos transformando a biologia do câncer de Pulmão. </t>
   </si>
   <si>
-    <t xml:space="preserve">Danielli Mathias</t>
+    <t xml:space="preserve">Danielli Mathias - RN</t>
   </si>
   <si>
     <t xml:space="preserve">14:35 - 15:05
@@ -231,7 +241,7 @@
   <si>
     <t xml:space="preserve">Mesa 5: Módulo doença avançada - pacientes com mutação driver 
 Presidente: Selem Asmar
-Moderadores:  Danielli Mathias , Leonardo Vila , Luiz José</t>
+Moderadores:  Danielli Mathias , Leonardo Vila , PET</t>
   </si>
   <si>
     <t xml:space="preserve">14:35 - 14:55
@@ -248,7 +258,7 @@
     <t xml:space="preserve">Toxicicidade Dermatologica pós tratamento </t>
   </si>
   <si>
-    <t>Jessica</t>
+    <t xml:space="preserve">Jessica Guido </t>
   </si>
   <si>
     <t xml:space="preserve">15:15 - 15:30</t>
@@ -273,9 +283,19 @@
 (40 minutos) </t>
   </si>
   <si>
-    <t xml:space="preserve">Mesa 6: Módulo doença avançada - Pacientes sem mutação driver 
-Presidente:   Sandra
-Moderadores: Nadja , Debora Porto</t>
+    <r>
+      <t xml:space="preserve">Mesa 6: Módulo doença avançada - Pacientes sem mutação driver 
+Presidente:   Sandra Oliveira
+Moderadores: Nadja Rolim  , Débora Porto, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="64"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve">Luiz José </t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">16:30 - 16:50
@@ -285,7 +305,8 @@
     <t xml:space="preserve">CASO CLINICO - Doença metastático</t>
   </si>
   <si>
-    <t xml:space="preserve">Vlad </t>
+    <t xml:space="preserve">Vladmir - SP 
+*online*</t>
   </si>
   <si>
     <t xml:space="preserve">16:50 - 17:10
@@ -299,7 +320,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="11.000000"/>
       <color indexed="64"/>
@@ -309,6 +330,15 @@
       <b/>
       <sz val="11.000000"/>
       <color indexed="64"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
@@ -415,7 +445,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -438,6 +468,12 @@
     <xf fontId="0" fillId="2" borderId="3" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="2" fillId="2" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="2" borderId="4" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -452,6 +488,12 @@
     </xf>
     <xf fontId="0" fillId="2" borderId="3" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="2" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="2" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1978,10 +2020,10 @@
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="9"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
@@ -3543,13 +3585,13 @@
       <c r="IT9" s="4"/>
     </row>
     <row r="10" ht="51" customHeight="1">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="9"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
@@ -3803,7 +3845,7 @@
       <c r="IT10" s="4"/>
     </row>
     <row r="11" ht="28.5" customHeight="1">
-      <c r="A11" s="9"/>
+      <c r="A11" s="11"/>
       <c r="B11" s="5" t="s">
         <v>23</v>
       </c>
@@ -4063,7 +4105,7 @@
       <c r="IT11" s="4"/>
     </row>
     <row r="12" ht="28.5" customHeight="1">
-      <c r="A12" s="10"/>
+      <c r="A12" s="12"/>
       <c r="B12" s="5" t="s">
         <v>25</v>
       </c>
@@ -4324,10 +4366,10 @@
       <c r="A13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="12"/>
+      <c r="C13" s="14"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
@@ -4584,10 +4626,10 @@
       <c r="A14" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="16"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
@@ -6672,10 +6714,10 @@
       <c r="A22" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="12"/>
+      <c r="C22" s="14"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
@@ -7194,10 +7236,10 @@
       <c r="A24" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="16"/>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
@@ -7716,7 +7758,7 @@
       <c r="A26" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="17" t="s">
         <v>56</v>
       </c>
       <c r="C26" s="5" t="s">
@@ -7978,10 +8020,10 @@
       <c r="A27" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C27" s="12"/>
+      <c r="C27" s="14"/>
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
@@ -9539,7 +9581,7 @@
       <c r="IT32" s="4"/>
     </row>
     <row r="33" ht="22.5" customHeight="1">
-      <c r="A33" s="14">
+      <c r="A33" s="18">
         <v>46197.715277777781</v>
       </c>
       <c r="B33" s="5" t="s">
@@ -9817,8 +9859,8 @@
     <mergeCell ref="B33:C33"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.59055118110236238" right="0.19685039370078738" top="0" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="67" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageMargins left="0.59055118110236238" right="0.19685039370078738" top="0.59499999999999997" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="63" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
Update session details and speaker names for Recife Tórax 2026
- Removed Ana Rita Carvalho from the list of moderators for Mesa 1.
- Updated speaker name from "Luiz Felipe" to "Luiz Felipe Carvalho" in the schedule.
- Revised moderator name from "Luiz José" to "Luiz José de Barros" for Mesa 6.
- Ensured consistency across HTML and CSV files with the latest changes.
</commit_message>
<xml_diff>
--- a/recifetorax2026/schedule/programacao-preliminar.xlsx
+++ b/recifetorax2026/schedule/programacao-preliminar.xlsx
@@ -66,7 +66,7 @@
   <si>
     <t xml:space="preserve">Mesa 1: Atualização em Fatores de Risco e Diagnóstico Precoce 
 Presidente: Alfredo Leite 
-Moderadores:   Leonardo Pontual ,  Antônio Douglas, Ana Rita Carvalho </t>
+Moderadores:   Leonardo Pontual ,  Antônio Douglas</t>
   </si>
   <si>
     <t xml:space="preserve">08:30 - 08:45 
@@ -130,7 +130,7 @@
     <t xml:space="preserve">Hugo Veiga</t>
   </si>
   <si>
-    <t xml:space="preserve">DISCUSSAO </t>
+    <t xml:space="preserve">DISCUSSÃO </t>
   </si>
   <si>
     <t xml:space="preserve">10:20 - 10:40
@@ -179,7 +179,7 @@
 (45 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">SIMPOSIO SATELITE ASTRAZENECA - Doença Iressecavel - PACIFIC/LAURA</t>
+    <t xml:space="preserve">SIMPOSIO SATELITE ASTRAZENECA - Doença Irressecável - PACIFIC/LAURA</t>
   </si>
   <si>
     <t xml:space="preserve">Victor Gondim - RJ</t>
@@ -248,14 +248,14 @@
 (20 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">Luiz Felipe </t>
+    <t xml:space="preserve">Luiz Felipe Carvalho </t>
   </si>
   <si>
     <t xml:space="preserve">14:55 - 15:15
 (20 min)</t>
   </si>
   <si>
-    <t xml:space="preserve">Toxicicidade Dermatologica pós tratamento </t>
+    <t xml:space="preserve">Toxicidade Dermatologica pós tratamento </t>
   </si>
   <si>
     <t xml:space="preserve">Jessica Guido </t>
@@ -295,6 +295,14 @@
         <rFont val="Aptos Narrow"/>
       </rPr>
       <t xml:space="preserve">Luiz José </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="64"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve">de Barros </t>
     </r>
   </si>
   <si>
@@ -4106,10 +4114,10 @@
     </row>
     <row r="12" ht="28.5" customHeight="1">
       <c r="A12" s="12"/>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="14"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
@@ -5410,10 +5418,10 @@
       <c r="A17" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="14"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
@@ -9324,10 +9332,10 @@
       <c r="A32" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C32" s="4"/>
+      <c r="C32" s="14"/>
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
@@ -9841,21 +9849,24 @@
       <c r="IT33" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="18">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="B33:C33"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
Add hero sponsors carousel and update schedule details for Recife Tórax 2026
- Introduced a new hero sponsors carousel in the HTML to showcase event sponsors with a scrolling animation.
- Updated the CSS for the sponsors carousel to enhance styling and responsiveness.
- Revised session details in the schedule, including moderator updates and session name changes for clarity.
- Added new sponsor logos in PNG format to the project for improved visibility and branding.
</commit_message>
<xml_diff>
--- a/recifetorax2026/schedule/programacao-preliminar.xlsx
+++ b/recifetorax2026/schedule/programacao-preliminar.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <r>
       <t xml:space="preserve">
@@ -66,7 +66,7 @@
   <si>
     <t xml:space="preserve">Mesa 1: Atualização em Fatores de Risco e Diagnóstico Precoce 
 Presidente: Alfredo Leite 
-Moderadores:   Leonardo Pontual ,  Antônio Douglas</t>
+Moderadores: Leonardo Pontual, Antônio Douglas, Paulo Almeida </t>
   </si>
   <si>
     <t xml:space="preserve">08:30 - 08:45 
@@ -112,25 +112,39 @@
     <t xml:space="preserve">09:30 - 09:40 (10 min)</t>
   </si>
   <si>
-    <t>Debate</t>
+    <t xml:space="preserve">DISCUSSÃO </t>
   </si>
   <si>
     <t xml:space="preserve">09:40 - 10:20
 (40 min)</t>
   </si>
   <si>
-    <t xml:space="preserve">Mesa 2: Doença localizada
+    <r>
+      <t xml:space="preserve">Mesa 2: Doença localizada
 Presidente: Bruno Pacheco 
-Moderadores:  José Fernando Prado,  Ricardo Machado, Gustavo Ferreira </t>
+Moderadores: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="2"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve">Ilka Rocha</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve">, Ricardo Machado, Gustavo Ferreira </t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">CASO CLINICO </t>
   </si>
   <si>
     <t xml:space="preserve">Hugo Veiga</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DISCUSSÃO </t>
   </si>
   <si>
     <t xml:space="preserve">10:20 - 10:40
@@ -140,15 +154,14 @@
     <t xml:space="preserve">Coffee break </t>
   </si>
   <si>
-    <t xml:space="preserve">10:40 - 11:50
-(01 hora e 
-10 min) 
+    <t xml:space="preserve">10:40 - 11:30
+(50 min) 
 </t>
   </si>
   <si>
     <t xml:space="preserve">Mesa 3 : DESAFIOS NA CIRURGIA 
-Presidente:  Tomás Béder 
-Moderadores:   Eriberto,  Paula Abreu e Lima,  France Anne Reinaldo </t>
+Presidente: Tomás Béder 
+Moderadores: Eriberto Marques, Paula Abreu e Lima, France Anne Reinaldo </t>
   </si>
   <si>
     <t xml:space="preserve">10:40 - 10:55
@@ -198,8 +211,8 @@
   <si>
     <r>
       <t xml:space="preserve">Mesa 4: Doença localmente - Irressecável  e Oligometastatica 
-Presidente: Petrúcio Sarmento 
-Moderadores:  Victor Gondim, Thiago Darlan, </t>
+Presidente: Filippe Gouvêa  
+Moderadores: Victor Gondim, Thiago Darlan, </t>
     </r>
     <r>
       <rPr>
@@ -232,23 +245,23 @@
     <t xml:space="preserve">SIMPÓSIO SATÉLITE JOHNSON  - Anticorpos biespecíficos transformando a biologia do câncer de Pulmão. </t>
   </si>
   <si>
-    <t xml:space="preserve">Danielli Mathias - RN</t>
+    <t xml:space="preserve">Danielli Matias - RN</t>
   </si>
   <si>
-    <t xml:space="preserve">14:35 - 15:05
-(40 min) </t>
+    <t xml:space="preserve">14:35 - 15:30
+(55 min) </t>
   </si>
   <si>
     <t xml:space="preserve">Mesa 5: Módulo doença avançada - pacientes com mutação driver 
-Presidente: Selem Asmar
-Moderadores:  Danielli Mathias , Leonardo Vila , PET</t>
+Presidente: José Fernando Prado
+Moderadores: Danielli Matias - RN, Leonardo Vila, Ana Rita Carvalho</t>
   </si>
   <si>
     <t xml:space="preserve">14:35 - 14:55
 (20 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">Luiz Felipe Carvalho </t>
+    <t xml:space="preserve">Luis Felipe Carvalho </t>
   </si>
   <si>
     <t xml:space="preserve">14:55 - 15:15
@@ -258,10 +271,12 @@
     <t xml:space="preserve">Toxicidade Dermatologica pós tratamento </t>
   </si>
   <si>
-    <t xml:space="preserve">Jessica Guido </t>
+    <t xml:space="preserve">Jéssica Guido 
+*Online*</t>
   </si>
   <si>
-    <t xml:space="preserve">15:15 - 15:30</t>
+    <t xml:space="preserve">15:15 - 15:30
+(15 min)</t>
   </si>
   <si>
     <t xml:space="preserve">15:30 - 15:50
@@ -328,7 +343,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="11.000000"/>
       <color indexed="64"/>
@@ -344,13 +359,8 @@
       <sz val="11.000000"/>
       <name val="Aptos Narrow"/>
     </font>
-    <font>
-      <sz val="11.000000"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -360,6 +370,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
       </patternFill>
     </fill>
   </fills>
@@ -453,7 +468,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -497,13 +512,10 @@
     <xf fontId="0" fillId="2" borderId="3" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="2" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="3" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="2" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="2" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="2" borderId="1" numFmtId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1237,13 +1249,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="12.949999999999999" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="1" width="13.6328125"/>
-    <col customWidth="1" min="2" max="2" style="1" width="78.90625"/>
-    <col customWidth="1" min="3" max="3" style="1" width="19.6328125"/>
-    <col customWidth="1" min="4" max="254" style="1" width="9.1796875"/>
-    <col min="255" max="16384" style="1" width="9.1796875"/>
+    <col customWidth="1" min="1" max="1" style="1" width="13.625"/>
+    <col customWidth="1" min="2" max="2" style="1" width="78.875"/>
+    <col customWidth="1" min="3" max="3" style="1" width="19.625"/>
+    <col customWidth="1" min="4" max="4" style="1" width="67.125"/>
+    <col customWidth="1" min="5" max="255" style="1" width="9.125"/>
+    <col min="256" max="16384" style="1" width="9.125"/>
   </cols>
   <sheetData>
     <row r="1" ht="49.5" customHeight="1">
@@ -1503,6 +1516,7 @@
       <c r="IR1" s="4"/>
       <c r="IS1" s="4"/>
       <c r="IT1" s="4"/>
+      <c r="IU1" s="4"/>
     </row>
     <row r="2" ht="28.5" customHeight="1">
       <c r="A2" s="5" t="s">
@@ -1763,6 +1777,7 @@
       <c r="IR2" s="4"/>
       <c r="IS2" s="4"/>
       <c r="IT2" s="4"/>
+      <c r="IU2" s="4"/>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="5" t="s">
@@ -2023,6 +2038,7 @@
       <c r="IR3" s="4"/>
       <c r="IS3" s="4"/>
       <c r="IT3" s="4"/>
+      <c r="IU3" s="4"/>
     </row>
     <row r="4" ht="51" customHeight="1">
       <c r="A4" s="5" t="s">
@@ -2283,6 +2299,7 @@
       <c r="IR4" s="4"/>
       <c r="IS4" s="4"/>
       <c r="IT4" s="4"/>
+      <c r="IU4" s="4"/>
     </row>
     <row r="5" ht="28.5" customHeight="1">
       <c r="A5" s="5" t="s">
@@ -2545,6 +2562,7 @@
       <c r="IR5" s="4"/>
       <c r="IS5" s="4"/>
       <c r="IT5" s="4"/>
+      <c r="IU5" s="4"/>
     </row>
     <row r="6" ht="28.5" customHeight="1">
       <c r="A6" s="5" t="s">
@@ -2807,6 +2825,7 @@
       <c r="IR6" s="4"/>
       <c r="IS6" s="4"/>
       <c r="IT6" s="4"/>
+      <c r="IU6" s="4"/>
     </row>
     <row r="7" ht="28.5" customHeight="1">
       <c r="A7" s="5" t="s">
@@ -3069,6 +3088,7 @@
       <c r="IR7" s="4"/>
       <c r="IS7" s="4"/>
       <c r="IT7" s="4"/>
+      <c r="IU7" s="4"/>
     </row>
     <row r="8" ht="28.5" customHeight="1">
       <c r="A8" s="5" t="s">
@@ -3331,6 +3351,7 @@
       <c r="IR8" s="4"/>
       <c r="IS8" s="4"/>
       <c r="IT8" s="4"/>
+      <c r="IU8" s="4"/>
     </row>
     <row r="9" ht="28.5" customHeight="1">
       <c r="A9" s="5" t="s">
@@ -3591,6 +3612,7 @@
       <c r="IR9" s="4"/>
       <c r="IS9" s="4"/>
       <c r="IT9" s="4"/>
+      <c r="IU9" s="4"/>
     </row>
     <row r="10" ht="51" customHeight="1">
       <c r="A10" s="10" t="s">
@@ -3851,6 +3873,7 @@
       <c r="IR10" s="4"/>
       <c r="IS10" s="4"/>
       <c r="IT10" s="4"/>
+      <c r="IU10" s="4"/>
     </row>
     <row r="11" ht="28.5" customHeight="1">
       <c r="A11" s="11"/>
@@ -4111,11 +4134,12 @@
       <c r="IR11" s="4"/>
       <c r="IS11" s="4"/>
       <c r="IT11" s="4"/>
+      <c r="IU11" s="4"/>
     </row>
     <row r="12" ht="28.5" customHeight="1">
       <c r="A12" s="12"/>
       <c r="B12" s="13" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="4"/>
@@ -4369,13 +4393,14 @@
       <c r="IR12" s="4"/>
       <c r="IS12" s="4"/>
       <c r="IT12" s="4"/>
+      <c r="IU12" s="4"/>
     </row>
     <row r="13" ht="28.5" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="4"/>
@@ -4629,15 +4654,16 @@
       <c r="IR13" s="4"/>
       <c r="IS13" s="4"/>
       <c r="IT13" s="4"/>
+      <c r="IU13" s="4"/>
     </row>
     <row r="14" ht="51" customHeight="1">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="16"/>
+      <c r="C14" s="9"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
@@ -4889,16 +4915,17 @@
       <c r="IR14" s="4"/>
       <c r="IS14" s="4"/>
       <c r="IT14" s="4"/>
+      <c r="IU14" s="4"/>
     </row>
     <row r="15" ht="28.5" customHeight="1">
       <c r="A15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
@@ -5151,16 +5178,17 @@
       <c r="IR15" s="4"/>
       <c r="IS15" s="4"/>
       <c r="IT15" s="4"/>
+      <c r="IU15" s="4"/>
     </row>
     <row r="16" ht="28.5" customHeight="1">
       <c r="A16" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>35</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
@@ -5413,13 +5441,14 @@
       <c r="IR16" s="4"/>
       <c r="IS16" s="4"/>
       <c r="IT16" s="4"/>
+      <c r="IU16" s="4"/>
     </row>
     <row r="17" ht="28.5" customHeight="1">
       <c r="A17" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="4"/>
@@ -5673,16 +5702,17 @@
       <c r="IR17" s="4"/>
       <c r="IS17" s="4"/>
       <c r="IT17" s="4"/>
+      <c r="IU17" s="4"/>
     </row>
     <row r="18" ht="28.5" customHeight="1">
       <c r="A18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
@@ -5935,13 +5965,14 @@
       <c r="IR18" s="4"/>
       <c r="IS18" s="4"/>
       <c r="IT18" s="4"/>
+      <c r="IU18" s="4"/>
     </row>
     <row r="19" ht="28.5" customHeight="1">
       <c r="A19" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -6195,13 +6226,14 @@
       <c r="IR19" s="4"/>
       <c r="IS19" s="4"/>
       <c r="IT19" s="4"/>
+      <c r="IU19" s="4"/>
     </row>
     <row r="20" ht="51" customHeight="1">
       <c r="A20" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -6455,16 +6487,17 @@
       <c r="IR20" s="4"/>
       <c r="IS20" s="4"/>
       <c r="IT20" s="4"/>
+      <c r="IU20" s="4"/>
     </row>
     <row r="21" ht="28.5" customHeight="1">
       <c r="A21" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
@@ -6717,13 +6750,14 @@
       <c r="IR21" s="4"/>
       <c r="IS21" s="4"/>
       <c r="IT21" s="4"/>
+      <c r="IU21" s="4"/>
     </row>
     <row r="22" ht="28.5" customHeight="1">
       <c r="A22" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="4"/>
@@ -6977,16 +7011,17 @@
       <c r="IR22" s="4"/>
       <c r="IS22" s="4"/>
       <c r="IT22" s="4"/>
+      <c r="IU22" s="4"/>
     </row>
     <row r="23" ht="28.5" customHeight="1">
       <c r="A23" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="C23" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>50</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
@@ -7239,15 +7274,16 @@
       <c r="IR23" s="4"/>
       <c r="IS23" s="4"/>
       <c r="IT23" s="4"/>
+      <c r="IU23" s="4"/>
     </row>
     <row r="24" ht="51" customHeight="1">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B24" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="C24" s="16"/>
+      <c r="C24" s="9"/>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
@@ -7499,16 +7535,17 @@
       <c r="IR24" s="4"/>
       <c r="IS24" s="4"/>
       <c r="IT24" s="4"/>
+      <c r="IU24" s="4"/>
     </row>
     <row r="25" ht="28.5" customHeight="1">
       <c r="A25" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
@@ -7761,16 +7798,17 @@
       <c r="IR25" s="4"/>
       <c r="IS25" s="4"/>
       <c r="IT25" s="4"/>
+      <c r="IU25" s="4"/>
     </row>
     <row r="26" ht="28.5" customHeight="1">
       <c r="A26" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="C26" s="15" t="s">
         <v>56</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>57</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
@@ -8023,13 +8061,14 @@
       <c r="IR26" s="4"/>
       <c r="IS26" s="4"/>
       <c r="IT26" s="4"/>
+      <c r="IU26" s="4"/>
     </row>
     <row r="27" ht="28.5" customHeight="1">
-      <c r="A27" s="5" t="s">
-        <v>58</v>
+      <c r="A27" s="15" t="s">
+        <v>57</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C27" s="14"/>
       <c r="D27" s="4"/>
@@ -8283,13 +8322,14 @@
       <c r="IR27" s="4"/>
       <c r="IS27" s="4"/>
       <c r="IT27" s="4"/>
+      <c r="IU27" s="4"/>
     </row>
     <row r="28" ht="28.5" customHeight="1">
       <c r="A28" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -8543,16 +8583,17 @@
       <c r="IR28" s="4"/>
       <c r="IS28" s="4"/>
       <c r="IT28" s="4"/>
+      <c r="IU28" s="4"/>
     </row>
     <row r="29" ht="28.5" customHeight="1">
       <c r="A29" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>62</v>
       </c>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
@@ -8805,13 +8846,14 @@
       <c r="IR29" s="4"/>
       <c r="IS29" s="4"/>
       <c r="IT29" s="4"/>
+      <c r="IU29" s="4"/>
     </row>
     <row r="30" ht="51" customHeight="1">
       <c r="A30" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -9065,16 +9107,17 @@
       <c r="IR30" s="4"/>
       <c r="IS30" s="4"/>
       <c r="IT30" s="4"/>
+      <c r="IU30" s="4"/>
     </row>
     <row r="31" ht="28.5" customHeight="1">
       <c r="A31" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>67</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
@@ -9327,13 +9370,14 @@
       <c r="IR31" s="4"/>
       <c r="IS31" s="4"/>
       <c r="IT31" s="4"/>
+      <c r="IU31" s="4"/>
     </row>
     <row r="32" ht="28.5" customHeight="1">
       <c r="A32" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C32" s="14"/>
       <c r="D32" s="4"/>
@@ -9587,13 +9631,14 @@
       <c r="IR32" s="4"/>
       <c r="IS32" s="4"/>
       <c r="IT32" s="4"/>
+      <c r="IU32" s="4"/>
     </row>
     <row r="33" ht="22.5" customHeight="1">
-      <c r="A33" s="18">
+      <c r="A33" s="17">
         <v>46197.715277777781</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
@@ -9847,6 +9892,7 @@
       <c r="IR33" s="4"/>
       <c r="IS33" s="4"/>
       <c r="IT33" s="4"/>
+      <c r="IU33" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="18">

</xml_diff>

<commit_message>
Update session details and moderators for Recife Tórax 2026 schedule
- Revised session headers in the HTML and CSV files to include additional moderators and updated session timings for clarity.
- Enhanced speaker details and session descriptions to reflect the latest changes in the program.
- Updated corresponding PDF and Excel files to ensure consistency across all schedule formats.
</commit_message>
<xml_diff>
--- a/recifetorax2026/schedule/programacao-preliminar.xlsx
+++ b/recifetorax2026/schedule/programacao-preliminar.xlsx
@@ -66,7 +66,7 @@
   <si>
     <t xml:space="preserve">Mesa 1: Atualização em Fatores de Risco e Diagnóstico Precoce 
 Presidente: Alfredo Leite 
-Moderadores: Leonardo Pontual, Antônio Douglas, Paulo Almeida </t>
+Moderadores: Leonardo Pontual, Antônio Douglas, Paulo Almeida, Maria Rosa Gomes  </t>
   </si>
   <si>
     <t xml:space="preserve">08:30 - 08:45 
@@ -119,26 +119,9 @@
 (40 min)</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Mesa 2: Doença localizada
+    <t xml:space="preserve">Mesa 2: Doença localizada
 Presidente: Bruno Pacheco 
-Moderadores: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color indexed="2"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t xml:space="preserve">Ilka Rocha</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t xml:space="preserve">, Ricardo Machado, Gustavo Ferreira </t>
-    </r>
+Moderadores: Ilka Rocha, Ricardo Machado, Gustavo Ferreira </t>
   </si>
   <si>
     <t xml:space="preserve">CASO CLINICO </t>
@@ -211,8 +194,8 @@
   <si>
     <r>
       <t xml:space="preserve">Mesa 4: Doença localmente - Irressecável  e Oligometastatica 
-Presidente: Filippe Gouvêa  
-Moderadores: Victor Gondim, Thiago Darlan, </t>
+Presidente: Rodrigo Arruda 
+Moderadores: Victor Gondim - RJ, Thiago Darlan, </t>
     </r>
     <r>
       <rPr>
@@ -238,33 +221,17 @@
 (20 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">13:55 - 14:35
-(40 min)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIMPÓSIO SATÉLITE JOHNSON  - Anticorpos biespecíficos transformando a biologia do câncer de Pulmão. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Danielli Matias - RN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14:35 - 15:30
-(55 min) </t>
+    <t xml:space="preserve">13:55 - 14:50
+(45 min) 
+</t>
   </si>
   <si>
     <t xml:space="preserve">Mesa 5: Módulo doença avançada - pacientes com mutação driver 
 Presidente: José Fernando Prado
-Moderadores: Danielli Matias - RN, Leonardo Vila, Ana Rita Carvalho</t>
+Moderadores: Danielli Matias - RN, Leonardo Vila, Ana Rita Carvalho, Jéssica Guido (online) </t>
   </si>
   <si>
-    <t xml:space="preserve">14:35 - 14:55
-(20 min) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luis Felipe Carvalho </t>
-  </si>
-  <si>
-    <t xml:space="preserve">14:55 - 15:15
+    <t xml:space="preserve">13:55 - 14:15
 (20 min)</t>
   </si>
   <si>
@@ -275,8 +242,25 @@
 *Online*</t>
   </si>
   <si>
-    <t xml:space="preserve">15:15 - 15:30
+    <t xml:space="preserve">14:15 - 14:35
+(20 min) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luis Felipe Carvalho </t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:35 - 14:50
 (15 min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:50 - 15:30
+(40 min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIMPÓSIO SATÉLITE JOHNSON &amp; JOHNSON  - Anticorpos biespecíficos transformando a biologia do câncer de Pulmão. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Danielli Matias - RN</t>
   </si>
   <si>
     <t xml:space="preserve">15:30 - 15:50
@@ -328,7 +312,7 @@
     <t xml:space="preserve">CASO CLINICO - Doença metastático</t>
   </si>
   <si>
-    <t xml:space="preserve">Vladmir - SP 
+    <t xml:space="preserve">Vladmir Lima  - SP 
 *online*</t>
   </si>
   <si>
@@ -1249,14 +1233,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="12.949999999999999" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="13" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="1" width="13.625"/>
-    <col customWidth="1" min="2" max="2" style="1" width="78.875"/>
-    <col customWidth="1" min="3" max="3" style="1" width="19.625"/>
-    <col customWidth="1" min="4" max="4" style="1" width="67.125"/>
-    <col customWidth="1" min="5" max="255" style="1" width="9.125"/>
-    <col min="256" max="16384" style="1" width="9.125"/>
+    <col customWidth="1" min="1" max="1" style="1" width="13.6328125"/>
+    <col customWidth="1" min="2" max="2" style="1" width="78.90625"/>
+    <col customWidth="1" min="3" max="3" style="1" width="19.6328125"/>
+    <col customWidth="1" min="4" max="4" style="1" width="67.08984375"/>
+    <col customWidth="1" min="5" max="255" style="1" width="9.08984375"/>
+    <col min="256" max="16384" style="1" width="9.08984375"/>
   </cols>
   <sheetData>
     <row r="1" ht="49.5" customHeight="1">
@@ -7013,16 +6997,14 @@
       <c r="IT22" s="4"/>
       <c r="IU22" s="4"/>
     </row>
-    <row r="23" ht="28.5" customHeight="1">
-      <c r="A23" s="5" t="s">
+    <row r="23" ht="51" customHeight="1">
+      <c r="A23" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>49</v>
-      </c>
+      <c r="C23" s="9"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
@@ -7276,14 +7258,16 @@
       <c r="IT23" s="4"/>
       <c r="IU23" s="4"/>
     </row>
-    <row r="24" ht="51" customHeight="1">
-      <c r="A24" s="15" t="s">
+    <row r="24" ht="28.5" customHeight="1">
+      <c r="A24" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="C24" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="C24" s="9"/>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
@@ -7801,15 +7785,13 @@
       <c r="IU25" s="4"/>
     </row>
     <row r="26" ht="28.5" customHeight="1">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="16" t="s">
-        <v>55</v>
+      <c r="B26" s="13" t="s">
+        <v>20</v>
       </c>
-      <c r="C26" s="15" t="s">
-        <v>56</v>
-      </c>
+      <c r="C26" s="14"/>
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
@@ -8064,13 +8046,15 @@
       <c r="IU26" s="4"/>
     </row>
     <row r="27" ht="28.5" customHeight="1">
-      <c r="A27" s="15" t="s">
+      <c r="A27" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B27" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C27" s="14"/>
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
@@ -9909,8 +9893,8 @@
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="B33:C33"/>

</xml_diff>